<commit_message>
Test with graph of iterations. A bit ugly
</commit_message>
<xml_diff>
--- a/decay.xlsx
+++ b/decay.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iba2016-my.sharepoint.com/personal/aiytx_goiba_net/Documents/Documents/Projects/Radioactive_decay/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="13_ncr:1_{216137BC-A3AB-4C46-941E-0557CB3B087C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32C62618-94A2-4569-95A7-970A81F6E0F3}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="13_ncr:1_{216137BC-A3AB-4C46-941E-0557CB3B087C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{603146A9-C444-4BC5-9308-51B0A1482306}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -765,7 +765,7 @@
       </c>
       <c r="G5" s="7"/>
       <c r="I5" s="18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" s="16" t="s">
         <v>15</v>

</xml_diff>